<commit_message>
data(preview): regenerate stats with the materialised npm universe
Byte-identical to the reviewed reference except the one broken row:
npm 'All tracked packages' now reads the real 2,572,386-package
universe (was 2, from the unmaterialised pointer).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KmfwrXQQwGkJ87EZCR1Xq
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -84293,7 +84293,7 @@
         </is>
       </c>
       <c r="C7" s="20" t="n">
-        <v>2</v>
+        <v>2572386</v>
       </c>
       <c r="D7" s="20" t="n">
         <v>849544</v>
@@ -84305,7 +84305,7 @@
         <v>30275</v>
       </c>
       <c r="G7" s="21" t="n">
-        <v>1174907</v>
+        <v>3747291</v>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data(preview): regenerate stats in the reviewed 3-table layout
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KmfwrXQQwGkJ87EZCR1Xq
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,10 +49,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="13"/>
     </font>
   </fonts>
   <fills count="10">
@@ -277,7 +273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -333,26 +329,15 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -84155,7 +84140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:M130"/>
+  <dimension ref="A2:M114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -84489,22 +84474,22 @@
     <row r="20">
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>Repo URLs</t>
+          <t>Outputs</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Class A</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Class B</t>
         </is>
       </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Class C</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
@@ -84758,1227 +84743,941 @@
       <c r="M33" s="37" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="39" t="inlineStr">
-        <is>
-          <t>Score distribution by component (scope 940)</t>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>Count</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="16" t="inlineStr">
-        <is>
-          <t>Component / subcomponent</t>
-        </is>
-      </c>
-      <c r="C37" s="40" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D37" s="17" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="E37" s="17" t="inlineStr">
-        <is>
-          <t>P25</t>
-        </is>
-      </c>
-      <c r="F37" s="17" t="inlineStr">
-        <is>
-          <t>P50</t>
-        </is>
-      </c>
-      <c r="G37" s="17" t="inlineStr">
-        <is>
-          <t>P75</t>
-        </is>
-      </c>
-      <c r="H37" s="18" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>GitHub repos (Class A)</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="n">
+        <v>915</v>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="41" t="inlineStr">
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>GitLab repos (Class A)</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>Total repos</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>Outputs</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="39" t="inlineStr">
         <is>
           <t>Concentration</t>
         </is>
       </c>
-      <c r="C38" s="42" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="D38" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="43" t="n">
-        <v>41</v>
-      </c>
-      <c r="F38" s="43" t="n">
-        <v>75</v>
-      </c>
-      <c r="G38" s="43" t="n">
-        <v>95</v>
-      </c>
-      <c r="H38" s="44" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>· bus factor</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>bf_commits_git_5y</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" s="21" t="n">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="19" t="inlineStr">
-        <is>
-          <t>· HHI</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>hhi_commits_git_5y</t>
-        </is>
-      </c>
-      <c r="D40" s="20" t="n">
-        <v>19</v>
-      </c>
-      <c r="E40" s="20" t="n">
-        <v>3060</v>
-      </c>
-      <c r="F40" s="20" t="n">
-        <v>5556</v>
-      </c>
-      <c r="G40" s="20" t="n">
-        <v>8987</v>
-      </c>
-      <c r="H40" s="21" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="41" t="inlineStr">
-        <is>
-          <t>Complexity</t>
-        </is>
-      </c>
-      <c r="C41" s="42" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="D41" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="43" t="n">
-        <v>26</v>
-      </c>
-      <c r="F41" s="43" t="n">
-        <v>49</v>
-      </c>
-      <c r="G41" s="43" t="n">
-        <v>73</v>
-      </c>
-      <c r="H41" s="44" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="19" t="inlineStr">
-        <is>
-          <t>· lines of code</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>loc_eoy</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="20" t="n">
-        <v>365</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>2704</v>
-      </c>
-      <c r="G42" s="20" t="n">
-        <v>21612</v>
-      </c>
-      <c r="H42" s="21" t="n">
-        <v>36990782</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="19" t="inlineStr">
-        <is>
-          <t>· cyclomatic max</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>cyclomatic_max</t>
-        </is>
-      </c>
-      <c r="D43" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="F43" s="20" t="n">
-        <v>18</v>
-      </c>
-      <c r="G43" s="20" t="n">
-        <v>48</v>
-      </c>
-      <c r="H43" s="21" t="n">
-        <v>12556</v>
+      <c r="C43" s="40" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="41" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="C44" s="42" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="D44" s="43" t="n">
-        <v>50</v>
-      </c>
-      <c r="E44" s="43" t="n">
-        <v>50</v>
-      </c>
-      <c r="F44" s="43" t="n">
-        <v>72</v>
-      </c>
-      <c r="G44" s="43" t="n">
-        <v>84</v>
-      </c>
-      <c r="H44" s="44" t="n">
-        <v>100</v>
+      <c r="B44" s="19" t="inlineStr">
+        <is>
+          <t>· Bus Factor (5 years, git contributors)</t>
+        </is>
+      </c>
+      <c r="C44" s="21" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>· OpenSSF score (0–10)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>openssf_score</t>
-        </is>
-      </c>
-      <c r="D45" s="30" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E45" s="30" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="F45" s="30" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G45" s="30" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="H45" s="29" t="n">
-        <v>9.6</v>
+          <t>· HHI (5 years, git contributors)</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="19" t="inlineStr">
-        <is>
-          <t>· CVE count 5y</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>cve_count_5y</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="21" t="n">
-        <v>10602</v>
+      <c r="B46" s="39" t="inlineStr">
+        <is>
+          <t>Complexity</t>
+        </is>
+      </c>
+      <c r="C46" s="40" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="41" t="inlineStr">
-        <is>
-          <t>Workload</t>
-        </is>
-      </c>
-      <c r="C47" s="42" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="D47" s="43" t="n">
-        <v>2</v>
-      </c>
-      <c r="E47" s="43" t="n">
-        <v>38</v>
-      </c>
-      <c r="F47" s="43" t="n">
-        <v>56</v>
-      </c>
-      <c r="G47" s="43" t="n">
-        <v>70</v>
-      </c>
-      <c r="H47" s="44" t="n">
-        <v>97</v>
+      <c r="B47" s="19" t="inlineStr">
+        <is>
+          <t>· Lines of Code (last year snapshot)</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>· LOC / contributor</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>loc_per_ac</t>
-        </is>
-      </c>
-      <c r="D48" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>107</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>302</v>
-      </c>
-      <c r="G48" s="20" t="n">
-        <v>804</v>
-      </c>
-      <c r="H48" s="21" t="n">
-        <v>353301</v>
+          <t>· Cyclomatic Complexity (last year snapshot)</t>
+        </is>
+      </c>
+      <c r="C48" s="21" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="19" t="inlineStr">
-        <is>
-          <t>· CVE / contributor</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>cve_per_ac</t>
-        </is>
-      </c>
-      <c r="D49" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="29" t="n">
-        <v>14</v>
+      <c r="B49" s="39" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C49" s="40" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>· net-new-issues / contributor</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>nni_per_ac</t>
-        </is>
-      </c>
-      <c r="D50" s="30" t="n">
-        <v>-9.93</v>
-      </c>
-      <c r="E50" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="30" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="G50" s="30" t="n">
+          <t>· OpenSSF Security Score (most recent data)</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="19" t="inlineStr">
+        <is>
+          <t>· CVE count (5 years)</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>Workload</t>
+        </is>
+      </c>
+      <c r="C52" s="40" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>· LOCs / active contributors (5 years)</t>
+        </is>
+      </c>
+      <c r="C53" s="21" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>· CVE / active contributors (5 years)</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>· Net new issues / active contributors (5 years)</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="C56" s="28" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Distribution</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="G59" s="18" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="39" t="inlineStr">
+        <is>
+          <t>Concentration</t>
+        </is>
+      </c>
+      <c r="C60" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="H50" s="29" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="45" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="C51" s="46" t="inlineStr">
-        <is>
-          <t>risk_score</t>
-        </is>
-      </c>
-      <c r="D51" s="47" t="n">
-        <v>11</v>
-      </c>
-      <c r="E51" s="47" t="n">
-        <v>44</v>
-      </c>
-      <c r="F51" s="47" t="n">
-        <v>54</v>
-      </c>
-      <c r="G51" s="47" t="n">
-        <v>65</v>
-      </c>
-      <c r="H51" s="48" t="n">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="39" t="inlineStr">
-        <is>
-          <t>Concentration funnel</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="16" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C55" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D55" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="19" t="inlineStr">
-        <is>
-          <t>input top repos</t>
-        </is>
-      </c>
-      <c r="C56" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D56" s="49" t="n">
+      <c r="D60" s="41" t="n">
+        <v>41</v>
+      </c>
+      <c r="E60" s="41" t="n">
+        <v>75</v>
+      </c>
+      <c r="F60" s="41" t="n">
+        <v>95</v>
+      </c>
+      <c r="G60" s="40" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>· Bus Factor (5 years, git contributors)</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="19" t="inlineStr">
-        <is>
-          <t>bus factor / HHI (git 5y) computed</t>
-        </is>
-      </c>
-      <c r="C57" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D57" s="49" t="n">
+      <c r="D61" s="20" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="19" t="inlineStr">
-        <is>
-          <t>bus factor / HHI (GitHub) computed</t>
-        </is>
-      </c>
-      <c r="C58" s="20" t="n">
-        <v>902</v>
-      </c>
-      <c r="D58" s="32" t="n">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="45" t="inlineStr">
-        <is>
-          <t>Concentration score</t>
-        </is>
-      </c>
-      <c r="C59" s="47" t="n">
-        <v>940</v>
-      </c>
-      <c r="D59" s="50" t="n">
+      <c r="E61" s="20" t="n">
         <v>1</v>
       </c>
+      <c r="F61" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="21" t="n">
+        <v>280</v>
+      </c>
     </row>
     <row r="62">
-      <c r="B62" s="39" t="inlineStr">
-        <is>
-          <t>Complexity funnel</t>
-        </is>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>· HHI (5 years, git contributors)</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="D62" s="20" t="n">
+        <v>3060</v>
+      </c>
+      <c r="E62" s="20" t="n">
+        <v>5556</v>
+      </c>
+      <c r="F62" s="20" t="n">
+        <v>8987</v>
+      </c>
+      <c r="G62" s="21" t="n">
+        <v>10000</v>
       </c>
     </row>
     <row r="63">
-      <c r="B63" s="16" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C63" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D63" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="B63" s="39" t="inlineStr">
+        <is>
+          <t>Complexity</t>
+        </is>
+      </c>
+      <c r="C63" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="41" t="n">
+        <v>26</v>
+      </c>
+      <c r="E63" s="41" t="n">
+        <v>49</v>
+      </c>
+      <c r="F63" s="41" t="n">
+        <v>73</v>
+      </c>
+      <c r="G63" s="40" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>input top repos</t>
+          <t>· Lines of Code (last year snapshot)</t>
         </is>
       </c>
       <c r="C64" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D64" s="49" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D64" s="20" t="n">
+        <v>365</v>
+      </c>
+      <c r="E64" s="20" t="n">
+        <v>2704</v>
+      </c>
+      <c r="F64" s="20" t="n">
+        <v>21612</v>
+      </c>
+      <c r="G64" s="21" t="n">
+        <v>36990782</v>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>lines of code (scc)</t>
+          <t>· Cyclomatic Complexity (last year snapshot)</t>
         </is>
       </c>
       <c r="C65" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D65" s="49" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D65" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="E65" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="F65" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="G65" s="21" t="n">
+        <v>12556</v>
       </c>
     </row>
     <row r="66">
-      <c r="B66" s="19" t="inlineStr">
-        <is>
-          <t>cyclomatic max (lizard)</t>
-        </is>
-      </c>
-      <c r="C66" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D66" s="49" t="n">
-        <v>1</v>
+      <c r="B66" s="39" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C66" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="D66" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="E66" s="41" t="n">
+        <v>72</v>
+      </c>
+      <c r="F66" s="41" t="n">
+        <v>84</v>
+      </c>
+      <c r="G66" s="40" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="19" t="inlineStr">
         <is>
-          <t>cognitive max (lizard)</t>
-        </is>
-      </c>
-      <c r="C67" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D67" s="49" t="n">
-        <v>1</v>
+          <t>· OpenSSF Security Score (most recent data)</t>
+        </is>
+      </c>
+      <c r="C67" s="30" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D67" s="30" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E67" s="30" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F67" s="30" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G67" s="29" t="n">
+        <v>9.6</v>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="19" t="inlineStr">
         <is>
-          <t>churn 5y</t>
+          <t>· CVE count (5 years)</t>
         </is>
       </c>
       <c r="C68" s="20" t="n">
-        <v>882</v>
-      </c>
-      <c r="D68" s="32" t="n">
-        <v>0.9379999999999999</v>
+        <v>0</v>
+      </c>
+      <c r="D68" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="21" t="n">
+        <v>10602</v>
       </c>
     </row>
     <row r="69">
-      <c r="B69" s="45" t="inlineStr">
-        <is>
-          <t>Complexity score</t>
-        </is>
-      </c>
-      <c r="C69" s="47" t="n">
+      <c r="B69" s="39" t="inlineStr">
+        <is>
+          <t>Workload</t>
+        </is>
+      </c>
+      <c r="C69" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="41" t="n">
+        <v>38</v>
+      </c>
+      <c r="E69" s="41" t="n">
+        <v>56</v>
+      </c>
+      <c r="F69" s="41" t="n">
+        <v>70</v>
+      </c>
+      <c r="G69" s="40" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>· LOCs / active contributors (5 years)</t>
+        </is>
+      </c>
+      <c r="C70" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="20" t="n">
+        <v>107</v>
+      </c>
+      <c r="E70" s="20" t="n">
+        <v>302</v>
+      </c>
+      <c r="F70" s="20" t="n">
+        <v>804</v>
+      </c>
+      <c r="G70" s="21" t="n">
+        <v>353301</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>· CVE / active contributors (5 years)</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="29" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="19" t="inlineStr">
+        <is>
+          <t>· Net new issues / active contributors (5 years)</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="n">
+        <v>-9.93</v>
+      </c>
+      <c r="D72" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="30" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F72" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="29" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="26" t="inlineStr">
+        <is>
+          <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="C73" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="D73" s="27" t="n">
+        <v>44</v>
+      </c>
+      <c r="E73" s="27" t="n">
+        <v>54</v>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>65</v>
+      </c>
+      <c r="G73" s="28" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="42" t="n"/>
+      <c r="B76" s="43" t="inlineStr">
+        <is>
+          <t>Stage 3: Eligibility</t>
+        </is>
+      </c>
+      <c r="C76" s="42" t="n"/>
+      <c r="D76" s="42" t="n"/>
+      <c r="E76" s="42" t="n"/>
+      <c r="F76" s="42" t="n"/>
+      <c r="G76" s="42" t="n"/>
+      <c r="H76" s="42" t="n"/>
+      <c r="I76" s="42" t="n"/>
+      <c r="J76" s="42" t="n"/>
+      <c r="K76" s="42" t="n"/>
+      <c r="L76" s="42" t="n"/>
+      <c r="M76" s="42" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="19" t="inlineStr">
+        <is>
+          <t>GitHub repos (Class A)</t>
+        </is>
+      </c>
+      <c r="C80" s="21" t="n">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="19" t="inlineStr">
+        <is>
+          <t>GitLab repos (Class A)</t>
+        </is>
+      </c>
+      <c r="C81" s="21" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="26" t="inlineStr">
+        <is>
+          <t>Total repos</t>
+        </is>
+      </c>
+      <c r="C82" s="28" t="n">
         <v>940</v>
       </c>
-      <c r="D69" s="50" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="39" t="inlineStr">
-        <is>
-          <t>Security funnel</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" s="16" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C73" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D73" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="19" t="inlineStr">
-        <is>
-          <t>input top repos</t>
-        </is>
-      </c>
-      <c r="C74" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D74" s="49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="19" t="inlineStr">
-        <is>
-          <t>OpenSSF score present</t>
-        </is>
-      </c>
-      <c r="C75" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D75" s="49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="19" t="inlineStr">
-        <is>
-          <t>CVE count 5y &gt; 0</t>
-        </is>
-      </c>
-      <c r="C76" s="20" t="n">
-        <v>208</v>
-      </c>
-      <c r="D76" s="32" t="n">
-        <v>0.221</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="19" t="inlineStr">
-        <is>
-          <t>OSS-Fuzz enrolled</t>
-        </is>
-      </c>
-      <c r="C77" s="20" t="n">
-        <v>135</v>
-      </c>
-      <c r="D77" s="32" t="n">
-        <v>0.144</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="19" t="inlineStr">
-        <is>
-          <t>CII Best Practices badge</t>
-        </is>
-      </c>
-      <c r="C78" s="20" t="n">
-        <v>31</v>
-      </c>
-      <c r="D78" s="32" t="n">
-        <v>0.033</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="45" t="inlineStr">
-        <is>
-          <t>Security score</t>
-        </is>
-      </c>
-      <c r="C79" s="47" t="n">
-        <v>940</v>
-      </c>
-      <c r="D79" s="50" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" s="39" t="inlineStr">
-        <is>
-          <t>Workload funnel</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="16" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C83" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D83" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="19" t="inlineStr">
-        <is>
-          <t>input top repos</t>
-        </is>
-      </c>
-      <c r="C84" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D84" s="49" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="85">
-      <c r="B85" s="19" t="inlineStr">
-        <is>
-          <t>issues data present</t>
-        </is>
-      </c>
-      <c r="C85" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D85" s="49" t="n">
-        <v>1</v>
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>Outputs</t>
+        </is>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" s="19" t="inlineStr">
         <is>
-          <t>per-AC ratios (loc/cve/nni) computed</t>
-        </is>
-      </c>
-      <c r="C86" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D86" s="49" t="n">
-        <v>1</v>
+          <t>Open Source</t>
+        </is>
+      </c>
+      <c r="C86" s="21" t="n">
+        <v>936</v>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="19" t="inlineStr">
         <is>
-          <t>issue_close_ratio computed</t>
-        </is>
-      </c>
-      <c r="C87" s="20" t="n">
-        <v>847</v>
-      </c>
-      <c r="D87" s="32" t="n">
-        <v>0.9009999999999999</v>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C87" s="21" t="n">
+        <v>918</v>
       </c>
     </row>
     <row r="88">
       <c r="B88" s="19" t="inlineStr">
         <is>
-          <t>issue_trend_score computed</t>
-        </is>
-      </c>
-      <c r="C88" s="20" t="n">
-        <v>642</v>
-      </c>
-      <c r="D88" s="32" t="n">
-        <v>0.6829999999999999</v>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="C88" s="21" t="n">
+        <v>736</v>
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="45" t="inlineStr">
-        <is>
-          <t>Workload score</t>
-        </is>
-      </c>
-      <c r="C89" s="47" t="n">
+      <c r="B89" s="19" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="C89" s="21" t="n">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="26" t="inlineStr">
+        <is>
+          <t>Eligibility checked</t>
+        </is>
+      </c>
+      <c r="C90" s="28" t="n">
         <v>940</v>
       </c>
-      <c r="D89" s="50" t="n">
+    </row>
+    <row r="93">
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>Distribution</t>
+        </is>
+      </c>
+      <c r="C93" s="17" t="inlineStr">
+        <is>
+          <t>Solo blocker</t>
+        </is>
+      </c>
+      <c r="D93" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E93" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="44" t="inlineStr">
+        <is>
+          <t>Open Source</t>
+        </is>
+      </c>
+      <c r="C94" s="45" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="51" t="n"/>
-      <c r="B92" s="52" t="inlineStr">
-        <is>
-          <t>Stage 3: Eligibility</t>
-        </is>
-      </c>
-      <c r="C92" s="51" t="n"/>
-      <c r="D92" s="51" t="n"/>
-      <c r="E92" s="51" t="n"/>
-      <c r="F92" s="51" t="n"/>
-      <c r="G92" s="51" t="n"/>
-      <c r="H92" s="51" t="n"/>
-      <c r="I92" s="51" t="n"/>
-      <c r="J92" s="51" t="n"/>
-      <c r="K92" s="51" t="n"/>
-      <c r="L92" s="51" t="n"/>
-      <c r="M92" s="51" t="n"/>
+      <c r="D94" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="E94" s="45" t="n">
+        <v>936</v>
+      </c>
+      <c r="F94" s="46" t="n">
+        <v>940</v>
+      </c>
     </row>
     <row r="95">
-      <c r="B95" s="39" t="inlineStr">
-        <is>
-          <t>Licenses (scope 940)</t>
-        </is>
+      <c r="B95" s="19" t="inlineStr">
+        <is>
+          <t>· License from manual override</t>
+        </is>
+      </c>
+      <c r="F95" s="21" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="96">
-      <c r="B96" s="16" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C96" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D96" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>· License from package registry</t>
+        </is>
+      </c>
+      <c r="F96" s="21" t="n">
+        <v>893</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="19" t="inlineStr">
         <is>
-          <t>input top repos (incl. archived)</t>
-        </is>
-      </c>
-      <c r="C97" s="20" t="n">
-        <v>940</v>
-      </c>
-      <c r="D97" s="49" t="n">
-        <v>1</v>
+          <t>· License from GitHub repo</t>
+        </is>
+      </c>
+      <c r="F97" s="21" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="19" t="inlineStr">
         <is>
-          <t>license resolved</t>
-        </is>
-      </c>
-      <c r="C98" s="20" t="n">
+          <t>· License from GitLab repo</t>
+        </is>
+      </c>
+      <c r="F98" s="21" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="44" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C99" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D99" s="45" t="n">
+        <v>22</v>
+      </c>
+      <c r="E99" s="45" t="n">
+        <v>918</v>
+      </c>
+      <c r="F99" s="46" t="n">
         <v>940</v>
-      </c>
-      <c r="D98" s="49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" s="19" t="inlineStr">
-        <is>
-          <t>· from override</t>
-        </is>
-      </c>
-      <c r="C99" s="20" t="n">
-        <v>23</v>
-      </c>
-      <c r="D99" s="32" t="n">
-        <v>0.024</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" s="19" t="inlineStr">
         <is>
-          <t>· from registry</t>
-        </is>
-      </c>
-      <c r="C100" s="20" t="n">
-        <v>893</v>
-      </c>
-      <c r="D100" s="32" t="n">
-        <v>0.95</v>
+          <t>· EOL (manual override)</t>
+        </is>
+      </c>
+      <c r="F100" s="21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="19" t="inlineStr">
         <is>
-          <t>· from GitHub</t>
-        </is>
-      </c>
-      <c r="C101" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="D101" s="32" t="n">
-        <v>0.01</v>
+          <t>· Archived (repo)</t>
+        </is>
+      </c>
+      <c r="F101" s="21" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="19" t="inlineStr">
         <is>
-          <t>· from GitLab</t>
-        </is>
-      </c>
-      <c r="C102" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="D102" s="32" t="n">
-        <v>0.016</v>
+          <t>· Archived but mirror-exempt</t>
+        </is>
+      </c>
+      <c r="F102" s="21" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="103">
-      <c r="B103" s="41" t="inlineStr">
-        <is>
-          <t>oss=True (OSS-approved)</t>
-        </is>
-      </c>
-      <c r="C103" s="43" t="n">
-        <v>936</v>
-      </c>
-      <c r="D103" s="53" t="n">
-        <v>0.996</v>
+      <c r="B103" s="44" t="inlineStr">
+        <is>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="C103" s="45" t="n">
+        <v>190</v>
+      </c>
+      <c r="D103" s="45" t="n">
+        <v>204</v>
+      </c>
+      <c r="E103" s="45" t="n">
+        <v>736</v>
+      </c>
+      <c r="F103" s="46" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="104">
       <c r="B104" s="19" t="inlineStr">
         <is>
-          <t>oss=False (known non-OSS)</t>
-        </is>
-      </c>
-      <c r="C104" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="D104" s="32" t="n">
-        <v>0.004</v>
+          <t>· GitHub Sponsors</t>
+        </is>
+      </c>
+      <c r="F104" s="21" t="n">
+        <v>376</v>
       </c>
     </row>
     <row r="105">
-      <c r="B105" s="23" t="inlineStr">
-        <is>
-          <t>oss unknown (no signal)</t>
-        </is>
-      </c>
-      <c r="C105" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D105" s="54" t="n">
-        <v>0</v>
+      <c r="B105" s="19" t="inlineStr">
+        <is>
+          <t>· FUNDING.yml</t>
+        </is>
+      </c>
+      <c r="F105" s="21" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="19" t="inlineStr">
+        <is>
+          <t>· funding.json</t>
+        </is>
+      </c>
+      <c r="F106" s="21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="19" t="inlineStr">
+        <is>
+          <t>· npm / PyPI funding field</t>
+        </is>
+      </c>
+      <c r="F107" s="21" t="n">
+        <v>215</v>
       </c>
     </row>
     <row r="108">
-      <c r="B108" s="39" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
+      <c r="B108" s="19" t="inlineStr">
+        <is>
+          <t>· Maintainer Sponsors</t>
+        </is>
+      </c>
+      <c r="F108" s="21" t="n">
+        <v>551</v>
       </c>
     </row>
     <row r="109">
-      <c r="B109" s="16" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C109" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D109" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
+      <c r="B109" s="19" t="inlineStr">
+        <is>
+          <t>· Open Collective</t>
+        </is>
+      </c>
+      <c r="F109" s="21" t="n">
+        <v>178</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="19" t="inlineStr">
         <is>
-          <t>eol (override)</t>
-        </is>
-      </c>
-      <c r="C110" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D110" s="32" t="n">
-        <v>0</v>
+          <t>· Institutional host / owner</t>
+        </is>
+      </c>
+      <c r="F110" s="21" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="111">
-      <c r="B111" s="19" t="inlineStr">
-        <is>
-          <t>archived</t>
-        </is>
-      </c>
-      <c r="C111" s="20" t="n">
-        <v>24</v>
-      </c>
-      <c r="D111" s="32" t="n">
-        <v>0.026</v>
+      <c r="B111" s="44" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="C111" s="45" t="n">
+        <v>59</v>
+      </c>
+      <c r="D111" s="45" t="n">
+        <v>60</v>
+      </c>
+      <c r="E111" s="45" t="n">
+        <v>880</v>
+      </c>
+      <c r="F111" s="46" t="n">
+        <v>940</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="19" t="inlineStr">
         <is>
-          <t>archived but mirror-exempt</t>
-        </is>
-      </c>
-      <c r="C112" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="D112" s="32" t="n">
-        <v>0.002</v>
+          <t>· Company-backed</t>
+        </is>
+      </c>
+      <c r="F112" s="21" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="113">
-      <c r="B113" s="45" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="C113" s="47" t="n">
-        <v>918</v>
-      </c>
-      <c r="D113" s="55" t="n">
-        <v>0.977</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="B116" s="39" t="inlineStr">
-        <is>
-          <t>Intent and nonprofit</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="B117" s="16" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C117" s="17" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D117" s="18" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" s="19" t="inlineStr">
-        <is>
-          <t>intent — any funding signal</t>
-        </is>
-      </c>
-      <c r="C118" s="20" t="n">
-        <v>736</v>
-      </c>
-      <c r="D118" s="32" t="n">
-        <v>0.7829999999999999</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="B119" s="19" t="inlineStr">
-        <is>
-          <t>intent — no funding signal</t>
-        </is>
-      </c>
-      <c r="C119" s="20" t="n">
-        <v>204</v>
-      </c>
-      <c r="D119" s="32" t="n">
-        <v>0.217</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="33" t="inlineStr">
-        <is>
-          <t>nonprofit — community / independent</t>
-        </is>
-      </c>
-      <c r="C120" s="34" t="n">
+      <c r="B113" s="19" t="inlineStr">
+        <is>
+          <t>· Community / independent</t>
+        </is>
+      </c>
+      <c r="F113" s="21" t="n">
         <v>880</v>
       </c>
-      <c r="D120" s="35" t="n">
-        <v>0.9359999999999999</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="B121" s="23" t="inlineStr">
-        <is>
-          <t>nonprofit — company-backed</t>
-        </is>
-      </c>
-      <c r="C121" s="24" t="n">
-        <v>60</v>
-      </c>
-      <c r="D121" s="54" t="n">
-        <v>0.064</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="B124" s="39" t="inlineStr">
-        <is>
-          <t>Eligibility rollup</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="B125" s="16" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="C125" s="17" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="D125" s="17" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E125" s="18" t="inlineStr">
-        <is>
-          <t>sole blocker</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="B126" s="19" t="inlineStr">
-        <is>
-          <t>oss</t>
-        </is>
-      </c>
-      <c r="C126" s="20" t="n">
-        <v>936</v>
-      </c>
-      <c r="D126" s="56" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="E126" s="21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="B127" s="19" t="inlineStr">
-        <is>
-          <t>intent</t>
-        </is>
-      </c>
-      <c r="C127" s="20" t="n">
-        <v>736</v>
-      </c>
-      <c r="D127" s="56" t="n">
-        <v>0.7829999999999999</v>
-      </c>
-      <c r="E127" s="21" t="n">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="B128" s="19" t="inlineStr">
-        <is>
-          <t>nonprofit</t>
-        </is>
-      </c>
-      <c r="C128" s="20" t="n">
-        <v>880</v>
-      </c>
-      <c r="D128" s="56" t="n">
-        <v>0.9359999999999999</v>
-      </c>
-      <c r="E128" s="21" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="B129" s="19" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="C129" s="20" t="n">
-        <v>918</v>
-      </c>
-      <c r="D129" s="56" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="E129" s="21" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="B130" s="26" t="inlineStr">
-        <is>
-          <t>eligible</t>
-        </is>
-      </c>
-      <c r="C130" s="27" t="n">
+    </row>
+    <row r="114">
+      <c r="B114" s="26" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="C114" s="47" t="n"/>
+      <c r="D114" s="27" t="n">
+        <v>275</v>
+      </c>
+      <c r="E114" s="27" t="n">
         <v>665</v>
       </c>
-      <c r="D130" s="57" t="n">
-        <v>0.7070000000000001</v>
-      </c>
-      <c r="E130" s="58" t="n"/>
+      <c r="F114" s="28" t="n">
+        <v>940</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data(preview): regenerate with the clarified Sponsors labels
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KmfwrXQQwGkJ87EZCR1Xq
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -85556,7 +85556,7 @@
     <row r="104">
       <c r="B104" s="19" t="inlineStr">
         <is>
-          <t>· GitHub Sponsors</t>
+          <t>· GitHub Sponsors (owner or repo)</t>
         </is>
       </c>
       <c r="F104" s="21" t="n">
@@ -85596,7 +85596,7 @@
     <row r="108">
       <c r="B108" s="19" t="inlineStr">
         <is>
-          <t>· Maintainer Sponsors</t>
+          <t>· GitHub Sponsors (maintainer)</t>
         </is>
       </c>
       <c r="F108" s="21" t="n">

</xml_diff>

<commit_message>
data(preview): regenerate with the fully-filled eligibility distribution
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KmfwrXQQwGkJ87EZCR1Xq
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -85451,6 +85451,15 @@
           <t>· License from manual override</t>
         </is>
       </c>
+      <c r="C95" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="D95" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="20" t="n">
+        <v>23</v>
+      </c>
       <c r="F95" s="21" t="n">
         <v>23</v>
       </c>
@@ -85461,6 +85470,15 @@
           <t>· License from package registry</t>
         </is>
       </c>
+      <c r="C96" s="20" t="n">
+        <v>889</v>
+      </c>
+      <c r="D96" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E96" s="20" t="n">
+        <v>889</v>
+      </c>
       <c r="F96" s="21" t="n">
         <v>893</v>
       </c>
@@ -85471,6 +85489,15 @@
           <t>· License from GitHub repo</t>
         </is>
       </c>
+      <c r="C97" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D97" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="20" t="n">
+        <v>9</v>
+      </c>
       <c r="F97" s="21" t="n">
         <v>9</v>
       </c>
@@ -85481,6 +85508,15 @@
           <t>· License from GitLab repo</t>
         </is>
       </c>
+      <c r="C98" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="D98" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="20" t="n">
+        <v>15</v>
+      </c>
       <c r="F98" s="21" t="n">
         <v>15</v>
       </c>
@@ -85510,6 +85546,15 @@
           <t>· EOL (manual override)</t>
         </is>
       </c>
+      <c r="C100" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="20" t="n">
+        <v>0</v>
+      </c>
       <c r="F100" s="21" t="n">
         <v>0</v>
       </c>
@@ -85520,6 +85565,15 @@
           <t>· Archived (repo)</t>
         </is>
       </c>
+      <c r="C101" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="D101" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="E101" s="20" t="n">
+        <v>2</v>
+      </c>
       <c r="F101" s="21" t="n">
         <v>24</v>
       </c>
@@ -85530,6 +85584,15 @@
           <t>· Archived but mirror-exempt</t>
         </is>
       </c>
+      <c r="C102" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="20" t="n">
+        <v>2</v>
+      </c>
       <c r="F102" s="21" t="n">
         <v>2</v>
       </c>
@@ -85559,6 +85622,15 @@
           <t>· GitHub Sponsors (owner or repo)</t>
         </is>
       </c>
+      <c r="C104" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="D104" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" s="20" t="n">
+        <v>376</v>
+      </c>
       <c r="F104" s="21" t="n">
         <v>376</v>
       </c>
@@ -85569,6 +85641,15 @@
           <t>· FUNDING.yml</t>
         </is>
       </c>
+      <c r="C105" s="20" t="n">
+        <v>31</v>
+      </c>
+      <c r="D105" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="20" t="n">
+        <v>391</v>
+      </c>
       <c r="F105" s="21" t="n">
         <v>391</v>
       </c>
@@ -85579,6 +85660,15 @@
           <t>· funding.json</t>
         </is>
       </c>
+      <c r="C106" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="20" t="n">
+        <v>8</v>
+      </c>
       <c r="F106" s="21" t="n">
         <v>8</v>
       </c>
@@ -85589,6 +85679,15 @@
           <t>· npm / PyPI funding field</t>
         </is>
       </c>
+      <c r="C107" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="20" t="n">
+        <v>215</v>
+      </c>
       <c r="F107" s="21" t="n">
         <v>215</v>
       </c>
@@ -85599,6 +85698,15 @@
           <t>· GitHub Sponsors (maintainer)</t>
         </is>
       </c>
+      <c r="C108" s="20" t="n">
+        <v>65</v>
+      </c>
+      <c r="D108" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="20" t="n">
+        <v>551</v>
+      </c>
       <c r="F108" s="21" t="n">
         <v>551</v>
       </c>
@@ -85609,6 +85717,15 @@
           <t>· Open Collective</t>
         </is>
       </c>
+      <c r="C109" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D109" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="20" t="n">
+        <v>178</v>
+      </c>
       <c r="F109" s="21" t="n">
         <v>178</v>
       </c>
@@ -85619,6 +85736,15 @@
           <t>· Institutional host / owner</t>
         </is>
       </c>
+      <c r="C110" s="20" t="n">
+        <v>47</v>
+      </c>
+      <c r="D110" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="20" t="n">
+        <v>90</v>
+      </c>
       <c r="F110" s="21" t="n">
         <v>90</v>
       </c>
@@ -85648,6 +85774,15 @@
           <t>· Company-backed</t>
         </is>
       </c>
+      <c r="C112" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="D112" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="E112" s="20" t="n">
+        <v>0</v>
+      </c>
       <c r="F112" s="21" t="n">
         <v>60</v>
       </c>
@@ -85657,6 +85792,15 @@
         <is>
           <t>· Community / independent</t>
         </is>
+      </c>
+      <c r="C113" s="20" t="n">
+        <v>880</v>
+      </c>
+      <c r="D113" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" s="20" t="n">
+        <v>880</v>
       </c>
       <c r="F113" s="21" t="n">
         <v>880</v>

</xml_diff>

<commit_message>
feat(stats): eligibility sub-row Solo = block-attribution, sorted by count
Redefine the sub-row Solo blocker as the sub-reason's share of its check's
sole-blocker total, so the sub-rows PARTITION the component (OSS: registry
1; Active: archived 10; Nonprofit: company-backed 59). Intent's signal
sub-rows read 0 — a present funding signal grants intent, never blocks, so
its 190 sole-blockers (zero signals) attach to no single signal row.
Sub-rows now sort by count descending; the two archived activity rows are
renamed 'Archived GitHub repo' / '... but mirror-exempt'.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KmfwrXQQwGkJ87EZCR1Xq
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -85448,77 +85448,77 @@
     <row r="95">
       <c r="B95" s="19" t="inlineStr">
         <is>
-          <t>· License from manual override</t>
+          <t>· License from package registry</t>
         </is>
       </c>
       <c r="C95" s="20" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D95" s="20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E95" s="20" t="n">
-        <v>23</v>
+        <v>889</v>
       </c>
       <c r="F95" s="21" t="n">
-        <v>23</v>
+        <v>893</v>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="19" t="inlineStr">
         <is>
-          <t>· License from package registry</t>
+          <t>· License from manual override</t>
         </is>
       </c>
       <c r="C96" s="20" t="n">
-        <v>889</v>
+        <v>0</v>
       </c>
       <c r="D96" s="20" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E96" s="20" t="n">
-        <v>889</v>
+        <v>23</v>
       </c>
       <c r="F96" s="21" t="n">
-        <v>893</v>
+        <v>23</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="19" t="inlineStr">
         <is>
-          <t>· License from GitHub repo</t>
+          <t>· License from GitLab repo</t>
         </is>
       </c>
       <c r="C97" s="20" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D97" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E97" s="20" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F97" s="21" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="19" t="inlineStr">
         <is>
-          <t>· License from GitLab repo</t>
+          <t>· License from GitHub repo</t>
         </is>
       </c>
       <c r="C98" s="20" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D98" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E98" s="20" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F98" s="21" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="99">
@@ -85543,45 +85543,45 @@
     <row r="100">
       <c r="B100" s="19" t="inlineStr">
         <is>
-          <t>· EOL (manual override)</t>
+          <t>· Archived GitHub repo</t>
         </is>
       </c>
       <c r="C100" s="20" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D100" s="20" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E100" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F100" s="21" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="19" t="inlineStr">
         <is>
-          <t>· Archived (repo)</t>
+          <t>· Archived GitHub repo but mirror-exempt</t>
         </is>
       </c>
       <c r="C101" s="20" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D101" s="20" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="E101" s="20" t="n">
         <v>2</v>
       </c>
       <c r="F101" s="21" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" s="19" t="inlineStr">
         <is>
-          <t>· Archived but mirror-exempt</t>
+          <t>· EOL (manual override)</t>
         </is>
       </c>
       <c r="C102" s="20" t="n">
@@ -85591,10 +85591,10 @@
         <v>0</v>
       </c>
       <c r="E102" s="20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F102" s="21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -85619,20 +85619,20 @@
     <row r="104">
       <c r="B104" s="19" t="inlineStr">
         <is>
-          <t>· GitHub Sponsors (owner or repo)</t>
+          <t>· GitHub Sponsors (maintainer)</t>
         </is>
       </c>
       <c r="C104" s="20" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D104" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E104" s="20" t="n">
-        <v>376</v>
+        <v>551</v>
       </c>
       <c r="F104" s="21" t="n">
-        <v>376</v>
+        <v>551</v>
       </c>
     </row>
     <row r="105">
@@ -85642,7 +85642,7 @@
         </is>
       </c>
       <c r="C105" s="20" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="D105" s="20" t="n">
         <v>0</v>
@@ -85657,7 +85657,7 @@
     <row r="106">
       <c r="B106" s="19" t="inlineStr">
         <is>
-          <t>· funding.json</t>
+          <t>· GitHub Sponsors (owner or repo)</t>
         </is>
       </c>
       <c r="C106" s="20" t="n">
@@ -85667,10 +85667,10 @@
         <v>0</v>
       </c>
       <c r="E106" s="20" t="n">
-        <v>8</v>
+        <v>376</v>
       </c>
       <c r="F106" s="21" t="n">
-        <v>8</v>
+        <v>376</v>
       </c>
     </row>
     <row r="107">
@@ -85695,58 +85695,58 @@
     <row r="108">
       <c r="B108" s="19" t="inlineStr">
         <is>
-          <t>· GitHub Sponsors (maintainer)</t>
+          <t>· Open Collective</t>
         </is>
       </c>
       <c r="C108" s="20" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="D108" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E108" s="20" t="n">
-        <v>551</v>
+        <v>178</v>
       </c>
       <c r="F108" s="21" t="n">
-        <v>551</v>
+        <v>178</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" s="19" t="inlineStr">
         <is>
-          <t>· Open Collective</t>
+          <t>· Institutional host / owner</t>
         </is>
       </c>
       <c r="C109" s="20" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D109" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E109" s="20" t="n">
-        <v>178</v>
+        <v>90</v>
       </c>
       <c r="F109" s="21" t="n">
-        <v>178</v>
+        <v>90</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" s="19" t="inlineStr">
         <is>
-          <t>· Institutional host / owner</t>
+          <t>· funding.json</t>
         </is>
       </c>
       <c r="C110" s="20" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="D110" s="20" t="n">
         <v>0</v>
       </c>
       <c r="E110" s="20" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="F110" s="21" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
     </row>
     <row r="111">
@@ -85771,39 +85771,39 @@
     <row r="112">
       <c r="B112" s="19" t="inlineStr">
         <is>
-          <t>· Company-backed</t>
+          <t>· Community / independent</t>
         </is>
       </c>
       <c r="C112" s="20" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="D112" s="20" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E112" s="20" t="n">
-        <v>0</v>
+        <v>880</v>
       </c>
       <c r="F112" s="21" t="n">
-        <v>60</v>
+        <v>880</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" s="19" t="inlineStr">
         <is>
-          <t>· Community / independent</t>
+          <t>· Company-backed</t>
         </is>
       </c>
       <c r="C113" s="20" t="n">
-        <v>880</v>
+        <v>59</v>
       </c>
       <c r="D113" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="E113" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E113" s="20" t="n">
-        <v>880</v>
-      </c>
       <c r="F113" s="21" t="n">
-        <v>880</v>
+        <v>60</v>
       </c>
     </row>
     <row r="114">

</xml_diff>

<commit_message>
data: regenerate from run-pipeline.sh stage-selection testing
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KmfwrXQQwGkJ87EZCR1Xq
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -85597,10 +85597,10 @@
         <v>0</v>
       </c>
       <c r="E107" s="20" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F107" s="21" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="108">

</xml_diff>

<commit_message>
data(overrides): point qca at KDE GitLab; drop redundant valid pins
qca now names its canonical home, invent.kde.org/libraries/qca (Debian's qca2
copyright Source, and Homebrew's head), instead of KDE's GitHub mirror — it
resolves to gl/kde-972. The mirror was only necessary because classify() did not
recognise invent.kde.org as GitLab; it now does.

The five no-git-upstream rows (jpeg, unzip, graphicsmagick, db, r) drop their
valid=False pins. Validity is derived, not declared: with no git_url there is no
git target to validate, so git_valid is False on its own.

Data regenerated by a full pipeline run; 83/83 health checks pass, 812 tests.
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -84345,10 +84345,10 @@
         <v>2771</v>
       </c>
       <c r="E21" s="20" t="n">
-        <v>6928</v>
+        <v>6927</v>
       </c>
       <c r="F21" s="20" t="n">
-        <v>10611</v>
+        <v>10610</v>
       </c>
       <c r="G21" s="32" t="n">
         <v>0.917</v>
@@ -84367,10 +84367,10 @@
         <v>225</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="F22" s="20" t="n">
-        <v>841</v>
+        <v>846</v>
       </c>
       <c r="G22" s="32" t="n">
         <v>0.073</v>
@@ -84389,10 +84389,10 @@
         <v>41</v>
       </c>
       <c r="E23" s="20" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F23" s="20" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G23" s="32" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
data: rebuild preview with the corrected components sheet
The `components` sheet now states the real OSS-approved set (the FSF arm was
missing) and credits workload's issue signal to both GitHub and GitLab.

83/83 health checks pass; board review verified consistent with the preview.
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -83848,7 +83848,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Maintenance burden per maintainer: LOC per active contributor, CVEs per active contributor, and net-new issues per active contributor (GitHub Issues Search, per-year opened − closed) — each percentile-ranked, combined by geometric mean. The divisor is the same 5-year active-contributor count concentration uses (AC = 0 scored as AC = 1).</t>
+          <t>Maintenance burden per maintainer: LOC per active contributor, CVEs per active contributor, and net-new issues per active contributor (GitHub Issues Search + GitLab issues API, merged by repo_id, per-year opened − closed) — each percentile-ranked, combined by geometric mean. The divisor is the same 5-year active-contributor count concentration uses (AC = 0 scored as AC = 1).</t>
         </is>
       </c>
     </row>
@@ -83872,7 +83872,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="62" customHeight="1">
+    <row r="20" ht="76" customHeight="1">
       <c r="B20" s="9" t="inlineStr">
         <is>
           <t>oss</t>
@@ -83880,7 +83880,7 @@
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>One SPDX license resolved per repo — manual override → registry license of the repo's packages → GitHub Licensee → GitLab API — then checked against the OSI-approved set (SPDX isOsiApproved ∪ curated extras). Expression-aware: 'mit OR apache-2.0' counts if any component is approved. Ternary: True / False / blank (unknown ≠ known-non-OSS).</t>
+          <t>One SPDX license resolved per repo — manual override → registry license of the repo's packages → GitHub Licensee → GitLab API — then checked against the approved set: SPDX isOsiApproved ∪ (isFsfLibre − content licenses) ∪ curated extras, so an FSF-libre software licence the OSI never formally reviewed still counts, while font/doc licences do not. Expression-aware: 'mit OR apache-2.0' counts if any component is approved. Ternary: True / False / blank (unknown ≠ known-non-OSS).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: gitlab repos gain the aliases column and three repo_ids
</commit_message>
<xml_diff>
--- a/data/preview/preview.xlsx
+++ b/data/preview/preview.xlsx
@@ -82516,10 +82516,10 @@
         <v>3559</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>1468</v>
+        <v>1465</v>
       </c>
       <c r="G11" s="28" t="n">
-        <v>11570</v>
+        <v>11567</v>
       </c>
     </row>
     <row r="14">
@@ -82645,10 +82645,10 @@
         <v>226</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="F22" s="20" t="n">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="G22" s="32" t="n">
         <v>0.073</v>
@@ -82689,10 +82689,10 @@
         <v>3016</v>
       </c>
       <c r="E24" s="34" t="n">
-        <v>7500</v>
+        <v>7497</v>
       </c>
       <c r="F24" s="34" t="n">
-        <v>11462</v>
+        <v>11459</v>
       </c>
       <c r="G24" s="35" t="n">
         <v>0.991</v>
@@ -82799,10 +82799,10 @@
         <v>535</v>
       </c>
       <c r="E29" s="20" t="n">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="F29" s="20" t="n">
-        <v>1468</v>
+        <v>1465</v>
       </c>
       <c r="G29" s="32" t="n">
         <v>0.127</v>
@@ -82821,10 +82821,10 @@
         <v>3038</v>
       </c>
       <c r="E30" s="27" t="n">
-        <v>7586</v>
+        <v>7583</v>
       </c>
       <c r="F30" s="27" t="n">
-        <v>11570</v>
+        <v>11567</v>
       </c>
       <c r="G30" s="36" t="n">
         <v>1</v>

</xml_diff>